<commit_message>
solegstar: Corrections in rev B3 and electronic-BOM
git-svn-id: svn://localhost/local-pentevo@1328 c6c76956-fad2-4150-a3a9-ea0a427205ba
</commit_message>
<xml_diff>
--- a/pcad/solegstar/01_rev_b3/zxevo_b3_bom.xlsx
+++ b/pcad/solegstar/01_rev_b3/zxevo_b3_bom.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Google_Drive\ZX\ZXEVO\rev.b\zxevo_revb3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\zxevo_revb3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFA22F7-9635-491E-A777-380C8B13A606}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="15180"/>
   </bookViews>
   <sheets>
     <sheet name="zxevo_pll_pal_eprom_ram_mod" sheetId="1" r:id="rId1"/>
@@ -460,12 +459,6 @@
     <t>TSOP44(50) II</t>
   </si>
   <si>
-    <t>GM71C18163C</t>
-  </si>
-  <si>
-    <t>IS41LV16100D, KM416C1204CT-5</t>
-  </si>
-  <si>
     <t>RS1, RS2</t>
   </si>
   <si>
@@ -719,17 +712,30 @@
   </si>
   <si>
     <t>Перечень элементов ZX-Evolution Revision B3</t>
+  </si>
+  <si>
+    <t>GM71C18163CT6</t>
+  </si>
+  <si>
+    <t>IS41С16100-50T(L), IC41C16100S, KM416C1204CT-5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="2">
@@ -926,7 +932,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -967,9 +973,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -990,6 +993,21 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1299,7 +1317,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K101"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1307,14 +1325,14 @@
     <col min="2" max="2" width="14.85546875" customWidth="1"/>
     <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="27.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.140625" customWidth="1"/>
     <col min="7" max="11" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1774,7 +1792,7 @@
         <v>58</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D23" s="12">
         <v>1</v>
@@ -2565,7 +2583,7 @@
       <c r="J59" s="5"/>
       <c r="K59" s="5"/>
     </row>
-    <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
         <v>140</v>
       </c>
@@ -2586,7 +2604,7 @@
       <c r="J60" s="5"/>
       <c r="K60" s="5"/>
     </row>
-    <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>141</v>
       </c>
@@ -2607,35 +2625,35 @@
       <c r="J61" s="5"/>
       <c r="K61" s="5"/>
     </row>
-    <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="10" t="s">
+    <row r="62" spans="1:11" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C62" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D62" s="12">
+      <c r="C62" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="D62" s="22">
         <v>2</v>
       </c>
-      <c r="E62" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
+      <c r="E62" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="19"/>
+      <c r="J62" s="19"/>
+      <c r="K62" s="19"/>
     </row>
     <row r="63" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C63" s="11" t="s">
         <v>138</v>
@@ -2653,13 +2671,13 @@
     </row>
     <row r="64" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="C64" s="11" t="s">
         <v>149</v>
-      </c>
-      <c r="B64" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="C64" s="11" t="s">
-        <v>151</v>
       </c>
       <c r="D64" s="12">
         <v>1</v>
@@ -2674,13 +2692,13 @@
     </row>
     <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>152</v>
-      </c>
-      <c r="B65" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="D65" s="12">
         <v>2</v>
@@ -2695,19 +2713,19 @@
     </row>
     <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="C66" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="11" t="s">
+      <c r="D66" s="12">
+        <v>1</v>
+      </c>
+      <c r="E66" s="14" t="s">
         <v>156</v>
-      </c>
-      <c r="C66" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="D66" s="12">
-        <v>1</v>
-      </c>
-      <c r="E66" s="15" t="s">
-        <v>158</v>
       </c>
       <c r="F66" s="5"/>
       <c r="G66" s="5"/>
@@ -2718,13 +2736,13 @@
     </row>
     <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C67" s="11" t="s">
         <v>159</v>
-      </c>
-      <c r="B67" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="C67" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="D67" s="12">
         <v>4</v>
@@ -2739,19 +2757,19 @@
     </row>
     <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D68" s="12">
         <v>1</v>
       </c>
-      <c r="E68" s="15" t="s">
-        <v>163</v>
+      <c r="E68" s="14" t="s">
+        <v>161</v>
       </c>
       <c r="F68" s="5"/>
       <c r="G68" s="5"/>
@@ -2762,13 +2780,13 @@
     </row>
     <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D69" s="12">
         <v>2</v>
@@ -2783,13 +2801,13 @@
     </row>
     <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C70" s="11" t="s">
         <v>166</v>
-      </c>
-      <c r="B70" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="C70" s="11" t="s">
-        <v>168</v>
       </c>
       <c r="D70" s="12">
         <v>1</v>
@@ -2804,13 +2822,13 @@
     </row>
     <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C71" s="11" t="s">
         <v>169</v>
-      </c>
-      <c r="B71" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="C71" s="11" t="s">
-        <v>171</v>
       </c>
       <c r="D71" s="12">
         <v>1</v>
@@ -2825,13 +2843,13 @@
     </row>
     <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C72" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="B72" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="C72" s="11" t="s">
-        <v>174</v>
       </c>
       <c r="D72" s="12">
         <v>1</v>
@@ -2846,13 +2864,13 @@
     </row>
     <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C73" s="11" t="s">
         <v>175</v>
-      </c>
-      <c r="B73" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="C73" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="D73" s="12">
         <v>1</v>
@@ -2867,13 +2885,13 @@
     </row>
     <row r="74" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C74" s="11" t="s">
         <v>178</v>
-      </c>
-      <c r="B74" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>180</v>
       </c>
       <c r="D74" s="12">
         <v>1</v>
@@ -2888,19 +2906,19 @@
     </row>
     <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C75" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="B75" s="11" t="s">
+      <c r="D75" s="12">
+        <v>1</v>
+      </c>
+      <c r="E75" s="13" t="s">
         <v>182</v>
-      </c>
-      <c r="C75" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="D75" s="12">
-        <v>1</v>
-      </c>
-      <c r="E75" s="13" t="s">
-        <v>184</v>
       </c>
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
@@ -2911,13 +2929,13 @@
     </row>
     <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C76" s="11" t="s">
         <v>185</v>
-      </c>
-      <c r="B76" s="11" t="s">
-        <v>186</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>187</v>
       </c>
       <c r="D76" s="12">
         <v>1</v>
@@ -2932,19 +2950,19 @@
     </row>
     <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="C77" s="11" t="s">
         <v>188</v>
-      </c>
-      <c r="B77" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="C77" s="11" t="s">
-        <v>190</v>
       </c>
       <c r="D77" s="12">
         <v>3</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F77" s="5"/>
       <c r="G77" s="5"/>
@@ -2955,13 +2973,13 @@
     </row>
     <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D78" s="12">
         <v>1</v>
@@ -2976,19 +2994,19 @@
     </row>
     <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="C79" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="D79" s="12">
+        <v>1</v>
+      </c>
+      <c r="E79" s="14" t="s">
         <v>194</v>
-      </c>
-      <c r="B79" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="C79" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="D79" s="12">
-        <v>1</v>
-      </c>
-      <c r="E79" s="15" t="s">
-        <v>196</v>
       </c>
       <c r="F79" s="5"/>
       <c r="G79" s="5"/>
@@ -2999,13 +3017,13 @@
     </row>
     <row r="80" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B80" s="11" t="s">
         <v>94</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D80" s="12">
         <v>1</v>
@@ -3020,13 +3038,13 @@
     </row>
     <row r="81" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D81" s="12">
         <v>1</v>
@@ -3041,19 +3059,19 @@
     </row>
     <row r="82" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="C82" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="B82" s="11" t="s">
+      <c r="D82" s="12">
+        <v>1</v>
+      </c>
+      <c r="E82" s="13" t="s">
         <v>202</v>
-      </c>
-      <c r="C82" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="D82" s="12">
-        <v>1</v>
-      </c>
-      <c r="E82" s="13" t="s">
-        <v>204</v>
       </c>
       <c r="F82" s="5"/>
       <c r="G82" s="5"/>
@@ -3064,19 +3082,19 @@
     </row>
     <row r="83" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D83" s="12">
         <v>1</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
@@ -3087,19 +3105,19 @@
     </row>
     <row r="84" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C84" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D84" s="12">
         <v>1</v>
       </c>
-      <c r="E84" s="15" t="s">
-        <v>208</v>
+      <c r="E84" s="14" t="s">
+        <v>206</v>
       </c>
       <c r="F84" s="5"/>
       <c r="G84" s="5"/>
@@ -3110,13 +3128,13 @@
     </row>
     <row r="85" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B85" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C85" s="11" t="s">
         <v>209</v>
-      </c>
-      <c r="B85" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="C85" s="11" t="s">
-        <v>211</v>
       </c>
       <c r="D85" s="12">
         <v>1</v>
@@ -3131,13 +3149,13 @@
     </row>
     <row r="86" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="C86" s="11" t="s">
         <v>212</v>
-      </c>
-      <c r="B86" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="C86" s="11" t="s">
-        <v>214</v>
       </c>
       <c r="D86" s="12">
         <v>1</v>
@@ -3152,13 +3170,13 @@
     </row>
     <row r="87" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D87" s="12">
         <v>1</v>
@@ -3173,13 +3191,13 @@
     </row>
     <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D88" s="12">
         <v>1</v>
@@ -3194,13 +3212,13 @@
     </row>
     <row r="89" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="B89" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C89" s="11" t="s">
         <v>219</v>
-      </c>
-      <c r="B89" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C89" s="11" t="s">
-        <v>221</v>
       </c>
       <c r="D89" s="12">
         <v>2</v>
@@ -3215,13 +3233,13 @@
     </row>
     <row r="90" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="C90" s="11" t="s">
         <v>222</v>
-      </c>
-      <c r="B90" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="C90" s="11" t="s">
-        <v>224</v>
       </c>
       <c r="D90" s="12">
         <v>1</v>
@@ -3236,13 +3254,13 @@
     </row>
     <row r="91" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D91" s="12">
         <v>1</v>
@@ -3256,19 +3274,19 @@
       <c r="K91" s="5"/>
     </row>
     <row r="92" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="16" t="s">
+      <c r="A92" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="B92" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="C92" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="B92" s="17" t="s">
-        <v>228</v>
-      </c>
-      <c r="C92" s="17" t="s">
-        <v>229</v>
-      </c>
-      <c r="D92" s="18">
-        <v>1</v>
-      </c>
-      <c r="E92" s="19"/>
+      <c r="D92" s="17">
+        <v>1</v>
+      </c>
+      <c r="E92" s="18"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
       <c r="H92" s="5"/>
@@ -3290,9 +3308,9 @@
       <c r="K93" s="5"/>
     </row>
     <row r="94" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="20"/>
-      <c r="B94" s="21"/>
-      <c r="C94" s="21"/>
+      <c r="A94" s="19"/>
+      <c r="B94" s="20"/>
+      <c r="C94" s="20"/>
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
@@ -3303,9 +3321,9 @@
       <c r="K94" s="5"/>
     </row>
     <row r="95" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="20"/>
-      <c r="B95" s="21"/>
-      <c r="C95" s="21"/>
+      <c r="A95" s="19"/>
+      <c r="B95" s="20"/>
+      <c r="C95" s="20"/>
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
@@ -3316,9 +3334,9 @@
       <c r="K95" s="5"/>
     </row>
     <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="20"/>
-      <c r="B96" s="21"/>
-      <c r="C96" s="21"/>
+      <c r="A96" s="19"/>
+      <c r="B96" s="20"/>
+      <c r="C96" s="20"/>
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="5"/>
@@ -3329,9 +3347,9 @@
       <c r="K96" s="5"/>
     </row>
     <row r="97" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="20"/>
-      <c r="B97" s="21"/>
-      <c r="C97" s="21"/>
+      <c r="A97" s="19"/>
+      <c r="B97" s="20"/>
+      <c r="C97" s="20"/>
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
@@ -3342,9 +3360,9 @@
       <c r="K97" s="5"/>
     </row>
     <row r="98" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="20"/>
-      <c r="B98" s="21"/>
-      <c r="C98" s="21"/>
+      <c r="A98" s="19"/>
+      <c r="B98" s="20"/>
+      <c r="C98" s="20"/>
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
@@ -3355,9 +3373,9 @@
       <c r="K98" s="5"/>
     </row>
     <row r="99" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="20"/>
-      <c r="B99" s="21"/>
-      <c r="C99" s="21"/>
+      <c r="A99" s="19"/>
+      <c r="B99" s="20"/>
+      <c r="C99" s="20"/>
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
@@ -3368,9 +3386,9 @@
       <c r="K99" s="5"/>
     </row>
     <row r="100" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="20"/>
-      <c r="B100" s="21"/>
-      <c r="C100" s="21"/>
+      <c r="A100" s="19"/>
+      <c r="B100" s="20"/>
+      <c r="C100" s="20"/>
       <c r="D100" s="5"/>
       <c r="E100" s="5"/>
       <c r="F100" s="5"/>
@@ -3381,9 +3399,9 @@
       <c r="K100" s="5"/>
     </row>
     <row r="101" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="20"/>
-      <c r="B101" s="21"/>
-      <c r="C101" s="21"/>
+      <c r="A101" s="19"/>
+      <c r="B101" s="20"/>
+      <c r="C101" s="20"/>
       <c r="D101" s="5"/>
       <c r="E101" s="5"/>
       <c r="F101" s="5"/>
@@ -3394,7 +3412,8 @@
       <c r="K101" s="5"/>
     </row>
   </sheetData>
-  <pageMargins left="0.70866141732283472" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>